<commit_message>
Leads: 2026-09-26 00:07 UTC (cycle 173)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -563,6 +563,66 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Rockland Builders</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>rockland-builders.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://rockland-builders.com/service-area/reading/</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Chester County</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>matthew@rocklandbuildersllc.net</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>610-641-9195</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Reading PA</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Reading PA</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 00:09 UTC (cycle 174)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -623,6 +623,238 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Rays Plumbing Service</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>raysplumbing.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://raysplumbing.com/water-heater-repair/</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Rays Plumbing</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>service@raysplumbing.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>(360) 667-7000</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Vancouver WA</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>100</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>water heater repair Vancouver WA</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>MAS Pro Service</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>masproservice.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://masproservice.com/water-heater-repair-installation-in-vancouver-wa/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Founded Founded</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>info@masproservice.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>360-907-3412</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Vancouver WA</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>90</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>water heater repair Vancouver WA</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>HVAC Service | Sheehe's Heating &amp; Home Improvements, Inc</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>sheehesheating.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://www.sheehesheating.com/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>sheehesheating88@gmail.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>(802) 342-0666</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Rutland VT</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>88</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>heating and cooling company Rutland VT</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>The Gas Doctors | Vermonts finest HVAC Technicians -</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>thegasdoctors.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://thegasdoctors.com/services/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>info@thegasdoctors.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>802-287-1765</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Rutland VT</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>76</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>heating and cooling company Rutland VT</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 00:12 UTC (cycle 176)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -764,7 +764,6 @@
           <t>https://www.sheehesheating.com/</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>sheehesheating88@gmail.com</t>
@@ -820,7 +819,6 @@
           <t>https://thegasdoctors.com/services/</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>info@thegasdoctors.com</t>
@@ -850,6 +848,66 @@
         </is>
       </c>
       <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>HEP Heat and Air Johnson City South</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>hepheatandair.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://hepheatandair.com/hep-heating-and-air-johnson-city-south</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Efficient Solutions</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>info@hepheatandair.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(423) 228-7742</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Johnson City TN</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>100</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>HVAC contractor Johnson City TN</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 00:17 UTC (cycle 180)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -913,6 +913,118 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Best Rooter Service</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>bestrooterservice.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://www.bestrooterservice.com/bellingham-drain-cleaning-services/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>admin@bestrooterservice.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(360) 738-8393</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Bellingham WA</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>90</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>drain cleaning service Bellingham WA</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Septic &amp; Drain</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>primeplumber24.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://primeplumber24.com/service/wa/bellingham/drain-cleaning</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Drain Cleaning</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>contact@primeplumber24.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Bellingham WA</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>86</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>drain cleaning service Bellingham WA</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 00:29 UTC (cycle 188)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -934,7 +934,6 @@
           <t>https://www.bestrooterservice.com/bellingham-drain-cleaning-services/</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>admin@bestrooterservice.com</t>
@@ -1000,7 +999,6 @@
           <t>contact@primeplumber24.com</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>Bellingham WA</t>
@@ -1020,6 +1018,118 @@
         </is>
       </c>
       <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>423 Roofing and Construction</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>423-roofing.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://423-roofing.com/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>george@423-roofing.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(214) 914 0550</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Denton TX</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>100</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>roofing contractor Denton TX</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Glory Roofing and Construction, Corp.</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>roofingglory.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://roofingglory.com/service-areas/denton</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Roofing Glory</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>info@roofingglory.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Denton TX</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>76</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>roofing contractor Denton TX</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 00:31 UTC (cycle 189)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1044,7 +1044,6 @@
           <t>https://423-roofing.com/</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>george@423-roofing.com</t>
@@ -1110,7 +1109,6 @@
           <t>info@roofingglory.com</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>Denton TX</t>
@@ -1130,6 +1128,66 @@
         </is>
       </c>
       <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Residential Roofers Tulsa, OK (Roof Replacement &amp; Repair) | Ranger Roofing of Ok</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>rangerroofingok.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://rangerroofingok.com/residential-roofing/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Inspection Enable</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>info@rangerroofingok.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>(918) 342-2222</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Tulsa OK</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>90</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>residential roofing company Tulsa OK</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 00:44 UTC (cycle 198)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1193,6 +1193,66 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Air Efficiency Heating &amp; Cooling Services LLC | Santa Fe, NM</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>airefficiencyhvac.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://airefficiencyhvac.com/ac-repair-santa-fe-nm/</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Santa Fe</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>office@airefficiencyhvac.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>505-522-0000</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Santa Fe NM</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>90</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>air conditioning repair Santa Fe NM</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 00:47 UTC (cycle 200)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1253,6 +1253,62 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Residential Roofing company Santa Ana (714) 924-3969</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>santaanaroofing.us</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://www.santaanaroofing.us/residential-roofing-santa-ana-ca</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>info@santaanaroofing.us</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>(714) 924-3969</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Santa Ana CA</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>98</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>residential roofing company Santa Ana CA</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 00:48 UTC (cycle 201)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1274,7 +1274,6 @@
           <t>https://www.santaanaroofing.us/residential-roofing-santa-ana-ca</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>info@santaanaroofing.us</t>
@@ -1304,6 +1303,126 @@
         </is>
       </c>
       <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Dauntless Roofing Systems</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>dauntlessroofingsystems.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://dauntlessroofingsystems.com/roofing-company-in-clearwater-fl/</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Pause Dauntless</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>info@dauntlessroofingsystems.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>(813) 550-1245</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Clearwater FL</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>100</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>residential roofing company Clearwater FL</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Eagle's Landing General Contracting</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>el-gc.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://el-gc.com/services/roof-replacement-richardson-tx/</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>North Texas</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>tim@el-gc.com</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>(972) 210-5148</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Richardson TX</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>90</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>roof replacement Richardson TX</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 00:50 UTC (cycle 202)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1428,6 +1428,62 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Still's HVAC</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>stillshvacservice.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://stillshvacservice.com/heat-pump/heat-pump-installation-replacement.html</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>todds@stillshvacservice.com</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>(410) 714-4822</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Annapolis MD</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>100</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>heat pump installation Annapolis MD</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 04:24 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1449,7 +1449,6 @@
           <t>https://stillshvacservice.com/heat-pump/heat-pump-installation-replacement.html</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>todds@stillshvacservice.com</t>
@@ -1479,6 +1478,66 @@
         </is>
       </c>
       <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Heat Pump Installation &amp; Repair Bellingham, WA | Comfort Zone HVAC</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>comfortzonehvacwhatcom.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://www.comfortzonehvacwhatcom.com/heat-pumps-repair-installation</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Aubrey Hofer</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>comfortzonehvac5@gmail.com</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>(360) 319-2996</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Bellingham WA</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>100</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>heat pump installation Bellingham WA</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 04:27 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1543,6 +1543,62 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>AJs Refrigeration</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>bestlocalrepair.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://bestlocalrepair.com/hvac-westminster/</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>galacticdiplomat@icloud.com</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>(720) 717-0050</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Westminster CO</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>90</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>HVAC contractor Westminster CO</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 04:32 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1564,7 +1564,6 @@
           <t>https://bestlocalrepair.com/hvac-westminster/</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>galacticdiplomat@icloud.com</t>
@@ -1594,6 +1593,126 @@
         </is>
       </c>
       <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Water Heater Repair in Sarasota, FL | Johnson &amp; Sons Plumbing</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>johnsonandsonsplumbingllc.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://www.johnsonandsonsplumbingllc.com/water-heater-repair-sarasota/</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Steve Johnson</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>johnsonandsonsplumbingllc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>(941) 879-6430</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Sarasota FL</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>100</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>water heater repair Sarasota FL</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Rising Son Plumbing</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>risingsonplumbingkansas.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://risingsonplumbingkansas.com/</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Service With</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>risingsonplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>785-917-1616</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Lawrence KS</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>100</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>water heater repair Lawrence KS</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 04:39 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1718,6 +1718,66 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>NEXGEN Roofing</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>nexgenfl.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://www.nexgenfl.com/roof-cost-jacksonville</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Brandon Cornellier</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>info@nexgenfl.com</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>(904) 802-7150</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>90</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>roof replacement Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 04:46 UTC (cycle 16)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1778,6 +1778,62 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Xtreme Roofing LLC.</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>xtremeroofingllc.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://xtremeroofingllc.com/</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>info@indiantypefoundry.com</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>228-263-0293</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Gulfport MS</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>96</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>roofing contractor Gulfport MS</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 04:55 UTC (cycle 22)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1799,7 +1799,6 @@
           <t>https://xtremeroofingllc.com/</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>info@indiantypefoundry.com</t>
@@ -1829,6 +1828,66 @@
         </is>
       </c>
       <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Dependable Plumber Inc</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>plumbercaliforniadpi.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://plumbercaliforniadpi.com/services/water-heater-repair</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Dependable Plumber</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>info@plumbercaliforniadpi.com</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>(951) 467-1115</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Moreno Valley CA</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>90</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>water heater repair Moreno Valley CA</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 05:03 UTC (cycle 28)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1893,6 +1893,66 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Rodeo Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>rodeoheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://rodeoheatingandcooling.com/</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Service Meet</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>rodeoheatingandcooling@gmail.com</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>602 313 1959</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>88</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>heating and cooling company Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 05:24 UTC (cycle 42)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1953,6 +1953,66 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Clearwater Roofing | King Roofing &amp; Sheet Metal</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>kingworksfl.com</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://kingworksfl.com/clearwater.html</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>King Roofing</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>office@kingworksfl.com</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>352-345-8810</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Clearwater FL</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>100</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Clearwater FL</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 05:28 UTC (cycle 45)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2013,6 +2013,66 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Plumber New Braunfels</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>plumbernewbraunfels.com</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://plumbernewbraunfels.com/</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>New Braunfels</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>mishiniazi44@gmail.com</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>(830) 215-9740</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>90</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>emergency plumber New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 05:37 UTC (cycle 51)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2073,6 +2073,126 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>A Drop Above Plumbing</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>adropaboveplumbing.com</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://www.adropaboveplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Reviews Trusted</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>adropaboveplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>847-461-3236</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Rockford IL</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>90</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>plumbing company Rockford IL</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>YB MECHANICAL LLC</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>ybmechanical.com</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://ybmechanical.com/water-heater-repair-waldorf-md/</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Prince George</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>info@ybmechanical.com</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>(833) 680-1132</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Waldorf MD</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>90</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>water heater repair Waldorf MD</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 05:38 UTC (cycle 52)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2193,6 +2193,126 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>All Seasons Professionals</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>allseasonsprohvac.com</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://allseasonsprohvac.com/hvac-contractors-tyler-tx/</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>East Texas</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>allseasonsprofessionals@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>903-962-3179</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Tyler TX</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>100</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>HVAC contractor Tyler TX</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Nailed-It Roofing</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>nailed-itroofing.com</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://www.nailed-itroofing.com/alpharetta-roofing/</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Why Alpharetta</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>info@nailed-itroofing.com</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>770-241-5648</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Alpharetta GA</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>90</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>roof repair company Alpharetta GA</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 05:54 UTC (cycle 63)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2313,6 +2313,126 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>A Plus Roofing Company - Richmond VA</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>aplusroofing.com</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://aplusroofing.com/metal-roofs/</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Leadership Team</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>info@a-plus-roofing.com</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>(804)-752-0008</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Richmond VA</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>98</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Richmond VA</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Emergency Plumber in Germantown, MD | 24/7 Plumbing Services</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>germantownmdplumbing.com</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>http://germantownmdplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>View All</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>info@germantownmdplumbing.com</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>(831) 215-0939</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Germantown MD</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>78</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>emergency plumber Germantown MD</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 05:57 UTC (cycle 65)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2433,6 +2433,62 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>lehiutahplumber.com</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>lehiutahplumber.com</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://lehiutahplumber.com/</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>office@lehiutahplumber.com</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>(385) 345-4458</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Lehi UT</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>90</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>plumber Lehi UT</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 06:03 UTC (cycle 69)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2454,7 +2454,6 @@
           <t>https://lehiutahplumber.com/</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
           <t>office@lehiutahplumber.com</t>
@@ -2484,6 +2483,66 @@
         </is>
       </c>
       <c r="L35" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Rite Now</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>callritenow.com</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://callritenow.com/heat-pumps/heat-pump-installation/</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Rite Now</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>info@ritenow.com</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>(940) 289-6816</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Denton TX</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>100</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>heat pump installation Denton TX</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 06:09 UTC (cycle 73)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2548,6 +2548,66 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>E.N.G. Roofing</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>engroofers.com</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://engroofers.com/areas-we-serve/katy-tx/roof-replacement/</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Wisconsin Wyoming</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>roofingsupport@engroofers.com</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>(346) 532-2997</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Katy TX</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>90</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>roof replacement Katy TX</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 06:11 UTC (cycle 74)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2608,6 +2608,66 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Benchmark Roofers</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>benchmarkroofers.com</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://benchmarkroofers.com/residential-roofing/</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Justin Woodworth</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>info@benchmarkroofers.com</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>(443) 454-1293</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Annapolis MD</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>90</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>residential roofing company Annapolis MD</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 06:18 UTC (cycle 79)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2668,6 +2668,66 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Aabco Roofing</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>aabcoroofing.co</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://aabcoroofing.co/areas-we-serve/west-palm-beach/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Metal Roofing</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>info@aabcoroofing.co</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>561-338-0608</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>West Palm Beach FL</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>100</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>metal roofing contractor West Palm Beach FL</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 06:21 UTC (cycle 81)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2728,6 +2728,62 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Reliable Plumbing in Wilmington, NC | Vantage Plumbing</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>vantageplumbing.net</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://www.vantageplumbing.net/</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>info@vantageplumbing.net</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>(910) 621-2607</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Wilmington NC</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>90</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>plumber Wilmington NC</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 06:22 UTC (cycle 82)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2749,7 +2749,6 @@
           <t>https://www.vantageplumbing.net/</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
           <t>info@vantageplumbing.net</t>
@@ -2779,6 +2778,66 @@
         </is>
       </c>
       <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Clear Home</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>clearhome.pro</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://clearhome.pro/services/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>New Orleans</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>hello@clearhome.pro</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>(504) 285-9060</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>New Orleans LA</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>100</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>metal roofing contractor New Orleans LA</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 06:34 UTC (cycle 90)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2843,6 +2843,62 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Pink Duck Plumbing</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>pinkduckplumbing.com</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://pinkduckplumbing.com/johnson-city-tn/drain-cleaning/</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>hello@pinkduckplumbing.com</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>(423) 732-3825</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Johnson City TN</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>90</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>drain cleaning service Johnson City TN</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 06:36 UTC (cycle 91)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2864,7 +2864,6 @@
           <t>https://pinkduckplumbing.com/johnson-city-tn/drain-cleaning/</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
           <t>hello@pinkduckplumbing.com</t>
@@ -2894,6 +2893,62 @@
         </is>
       </c>
       <c r="L42" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Residential Roofing | Fort Smith, AR | Elite Roofing</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>eliteroofingar.com</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://www.eliteroofingar.com/residential-services</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>eliteroofing@eliteroofingar.com</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>479-478-8668</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Fort Smith AR</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>90</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>residential roofing company Fort Smith AR</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 06:39 UTC (cycle 93)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2919,7 +2919,6 @@
           <t>https://www.eliteroofingar.com/residential-services</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
           <t>eliteroofing@eliteroofingar.com</t>
@@ -2949,6 +2948,66 @@
         </is>
       </c>
       <c r="L43" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Winding River Construction</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>windingriverconstruction.com</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://www.windingriverconstruction.com/roof-repair-parma/</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Fully Insured</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>info@windingrc.com</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>(216)816-7475</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Parma OH</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>90</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>roof repair company Parma OH</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 06:52 UTC (cycle 102)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3013,6 +3013,66 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Alpha HVAC Nashville</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>alphahvacnashville.com</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://alphahvacnashville.com/heat-pump-repair-installation/</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Why Nashville</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>info@alphahvacnashville.com</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>(615) 552-1922</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Nashville TN</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>80</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>heat pump installation Nashville TN</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 06:56 UTC (cycle 105)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L45"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3073,6 +3073,186 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Triple R Custom Metal Roofing - Fort Worth Roofing Services</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>triplercustommetalroofing.com</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>https://triplercustommetalroofing.com/</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Roofing Replacement</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>gregr@triplercustommetals.com</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>1817506955</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Fort Worth TX</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>100</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Fort Worth TX</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Roof Replacement &amp; Installation in Spokane, WA | Avidus</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>avidusroofingllc.com</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://avidusroofingllc.com/roof-replacement/</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Schedule Your</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>john@doe.com</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>(509) 230-0632</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Spokane WA</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>100</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>roof replacement Spokane WA</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>All Terrain Roofing</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>allterrainroofingcontractor.com</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>https://www.allterrainroofingcontractor.com/roof-replacement/</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Inland Northwest</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>tb111084@gmail.com</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>509-499-4643</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Spokane WA</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>90</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>roof replacement Spokane WA</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 07:02 UTC (cycle 109)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3253,6 +3253,66 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>JC Roofing</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>jcroofingfw.com</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>https://jcroofingfw.com/</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Family Trade</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>office@jcroofingtexas.com</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>(817) 318-7663</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Fort Worth TX</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>100</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>roofing contractor Fort Worth TX</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 07:05 UTC (cycle 111)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3313,6 +3313,66 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Eden Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>edenheatingandair.com</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>https://www.edenheatingandair.com/hvac/heat-pump-installation-replacement-lexington-ky</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Central Kentucky</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>info@edenheatingandair.com</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>(859) 314-0196</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Lexington KY</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>90</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>heat pump installation Lexington KY</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 07:06 UTC (cycle 112)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L50"/>
+  <dimension ref="A1:L51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3373,6 +3373,66 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Green Bay Hvac Pros</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>greenbayhvacpros.com</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>https://greenbayhvacpros.com/</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Green Bay</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>info@green-bayhvac.com</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>(920) 555-0349</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Green Bay WI</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>90</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>HVAC contractor Green Bay WI</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 07:08 UTC (cycle 113)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:L52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3433,6 +3433,62 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Summit Heating, A/C, Plumbing &amp; Electrical</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>summitheatingco.com</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>https://summitheatingco.com/hvac-arvada-co/</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>inquiries@summitheatingco.com</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>(720) 870-1580</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Arvada CO</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>90</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>HVAC contractor Arvada CO</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 07:09 UTC (cycle 114)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L52"/>
+  <dimension ref="A1:L53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3454,7 +3454,6 @@
           <t>https://summitheatingco.com/hvac-arvada-co/</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
           <t>inquiries@summitheatingco.com</t>
@@ -3484,6 +3483,62 @@
         </is>
       </c>
       <c r="L52" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>NexDrain Plumbing &amp; Drain</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>nexdrainplumbing.net</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>https://nexdrainplumbing.net/service-areas/irving-tx/drain-cleaning/</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>office@nexdrainplumbing.net</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>817-675-2239</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Irving TX</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>100</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>drain cleaning service Irving TX</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 07:19 UTC (cycle 121)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L53"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3509,7 +3509,6 @@
           <t>https://nexdrainplumbing.net/service-areas/irving-tx/drain-cleaning/</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
           <t>office@nexdrainplumbing.net</t>
@@ -3539,6 +3538,62 @@
         </is>
       </c>
       <c r="L53" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>AC Repair in Akron, OH | Echols Heating &amp; Air Conditioning, Inc.</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>echolsheating.com</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>https://www.echolsheating.com/air-conditioning-repair-akron</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>office@echolsheating.com</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>(234) 248-2777</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Akron OH</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>90</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>air conditioning repair Akron OH</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 07:28 UTC (cycle 127)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L54"/>
+  <dimension ref="A1:L55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3564,7 +3564,6 @@
           <t>https://www.echolsheating.com/air-conditioning-repair-akron</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
           <t>office@echolsheating.com</t>
@@ -3594,6 +3593,66 @@
         </is>
       </c>
       <c r="L54" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Barney's Plumbing LLC</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>barneysplumbingllc.com</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>https://barneysplumbingllc.com/kent/kent-sewer-services/sewer-repair/</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Bonney Lake</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>david@barneysplumbingllc.com</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>(253) 498-5434</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Kent WA</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>100</v>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>sewer repair Kent WA</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 07:34 UTC (cycle 131)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L55"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3658,6 +3658,66 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Bigfoot Plumbing</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>bigfootplumbingpnw.com</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>https://bigfootplumbingpnw.com/service-areas/gresham</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Glance Owner</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>contact@bigfootplumbingpnw.com</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>(971) 299-6800</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Gresham OR</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>90</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>plumber Gresham OR</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 07:44 UTC (cycle 138)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:L57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3718,6 +3718,66 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Drain Cleaning Concord NC | Piedmont Plumbing</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>piedmontplumbingnc.com</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>https://piedmontplumbingnc.com/drain-cleaning-services</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Connect Trusted</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>garya@piedmontplumbingnc.com</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>(980)-369-2035</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Concord NC</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>90</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>drain cleaning service Concord NC</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 08:13 UTC (cycle 158)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3778,6 +3778,66 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>ironandoakroofing.com</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>ironandoakroofing.com</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>https://ironandoakroofing.com/roofing-contractor-macon-ga-roof-repair-replacement/</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>South Georgia</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>office@ironandoakroofing.com</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>229-406-0539</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Macon GA</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>90</v>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>roof replacement Macon GA</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 08:19 UTC (cycle 162)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L58"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3838,6 +3838,66 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>HVAC Service in Arlington TX | 24/7 AC Repair &amp; Install</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>txairmechanics.com</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>https://www.txairmechanics.com/service-area/arlington</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Testimonials Trusted</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>info@txairmechanics.com</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>(817) 730-9344</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Arlington TX</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>100</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>HVAC contractor Arlington TX</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 08:29 UTC (cycle 169)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3898,6 +3898,122 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Red Tulip Plumbing</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>redtulipplumbing.com</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>https://www.redtulipplumbing.com/emergency-plumbing-services-in-fremont-ca/</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Call Us</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>redtulipplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>(510) 730-4957</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Fremont CA</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>100</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>emergency plumber Fremont CA</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Atlas Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>atlasheatingcooling.com</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>https://atlasheatingcooling.com/service-areas/troy-mi/</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>atlasair@live.com</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>(586) 339-4828</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Troy MI</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>100</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>heating and cooling company Troy MI</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 08:33 UTC (cycle 172)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:L62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3979,7 +3979,6 @@
           <t>https://atlasheatingcooling.com/service-areas/troy-mi/</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
           <t>atlasair@live.com</t>
@@ -4009,6 +4008,66 @@
         </is>
       </c>
       <c r="L61" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Home - Joe Ganzel Plumbing, Inc. -</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>jganzelplbg.com</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>https://jganzelplbg.com/</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Joe Ganzel</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>ganzelplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>419-865-6512</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Toledo OH</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>76</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>plumbing company Toledo OH</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 08:36 UTC (cycle 174)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L62"/>
+  <dimension ref="A1:L63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4073,6 +4073,66 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Metal Roofing in Kissimmee, FL | Matata Roofing</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>matataroofing.com</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>https://matataroofing.com/roofing/kissimmee/metal-roofing</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>For Florida</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>info@matataroofing.com</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>(321) 444-5191</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Kissimmee FL</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>80</v>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Kissimmee FL</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 08:49 UTC (cycle 183)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L63"/>
+  <dimension ref="A1:L64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4133,6 +4133,66 @@
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Hoffman Energy</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>hoffmanenergy.com</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>https://www.hoffmanenergy.com/locations/danbury/</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>General Manager</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>info@hoffmanenergy.com</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>877.359.0623</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Danbury CT</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>90</v>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>furnace repair Danbury CT</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 08:57 UTC (cycle 188)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L64"/>
+  <dimension ref="A1:L65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4193,6 +4193,62 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Water heater repair in Pearland</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>texasplumbingspecialists.com</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>https://texasplumbingspecialists.com/locations/pearland-tx/water-heater-repair</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>info@texasplumbingspecialists.com</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>(346) 908-9709</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Pearland TX</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>90</v>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>water heater repair Pearland TX</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 09:14 UTC (cycle 200)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L65"/>
+  <dimension ref="A1:L66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4214,7 +4214,6 @@
           <t>https://texasplumbingspecialists.com/locations/pearland-tx/water-heater-repair</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
           <t>info@texasplumbingspecialists.com</t>
@@ -4244,6 +4243,66 @@
         </is>
       </c>
       <c r="L65" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Penn Air Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>pennairhvac.com</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>https://pennairhvac.com/</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Book Online</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>info@pennairhvac.com</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>(717) 836-4575</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Harrisburg PA</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>90</v>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>heating and cooling company Harrisburg PA</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 12:54 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L66"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4308,6 +4308,122 @@
         </is>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Air Bourne Air Conditioning Heating and Indoor Air Quality</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>airbourneairinc.com</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>https://www.airbourneairinc.com/</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>davidf@airborneair.com</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>(281) 242-1245</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Katy TX</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>100</v>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>heating and cooling company Katy TX</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Koala Coolin</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>koalacoolin.com</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>https://www.koalacoolin.com/locations/pembroke-pines</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Real Google</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>contact@koalacoolin.com</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>(754) 282-7082</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Pembroke Pines FL</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>90</v>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>AC installation Pembroke Pines FL</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 12:58 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L68"/>
+  <dimension ref="A1:L69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4329,7 +4329,6 @@
           <t>https://www.airbourneairinc.com/</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
           <t>davidf@airborneair.com</t>
@@ -4419,6 +4418,66 @@
         </is>
       </c>
       <c r="L68" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Simi Heating &amp; Air, Inc.</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>airsimi.com</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>https://airsimi.com/</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Stu Pidasso</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>bsimi@airsimi.com</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>(209) 321-2001</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Stockton CA</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>80</v>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>HVAC contractor Stockton CA</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 13:00 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L69"/>
+  <dimension ref="A1:L70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4483,6 +4483,66 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Spangler Roofing | St. Petersburg's Family Roofer Since 1989</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>spanglerroofingllc.com</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>https://spanglerroofingllc.com/</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Roofing St</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>spanglerroof@gmail.com</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>(727) 397-3800</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>St Petersburg FL</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>80</v>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>roofing contractor St Petersburg FL</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 13:04 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L70"/>
+  <dimension ref="A1:L71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4543,6 +4543,66 @@
         </is>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Rc Sky Roofing Torrance ca</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>roofingtorranceca.com</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>https://roofingtorranceca.com/</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Roofing Torrance</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>roofingtorranceca0@gmail.com</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>(424) 540-2268</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Torrance CA</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>90</v>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>roofing contractor Torrance CA</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 13:12 UTC (cycle 15)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L71"/>
+  <dimension ref="A1:L72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4603,6 +4603,62 @@
         </is>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Professional Drain Service</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>professionaldrainofmobile.com</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>https://professionaldrainofmobile.com/</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>info@ndiscovered.com</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>(251) 645-2216</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Mobile AL</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>84</v>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>drain cleaning service Mobile AL</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 13:15 UTC (cycle 17)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L72"/>
+  <dimension ref="A1:L73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4624,7 +4624,6 @@
           <t>https://professionaldrainofmobile.com/</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
           <t>info@ndiscovered.com</t>
@@ -4654,6 +4653,66 @@
         </is>
       </c>
       <c r="L72" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>All In One General Contractor Inc</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>allinonegeneralcontractor.com</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>https://allinonegeneralcontractor.com/services/hvac-air-conditioning-repair-installation-silver-spring-md/</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Silver Spring</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>management@allinonegeneralcontractor.com</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>3014791115</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Silver Spring MD</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>100</v>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>air conditioning repair Silver Spring MD</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 13:16 UTC (cycle 18)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L73"/>
+  <dimension ref="A1:L74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4718,6 +4718,66 @@
         </is>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Larson &amp; Keeney Home Services</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>larsonhomeservices.com</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>https://www.larsonhomeservices.com/service-area/rochester-mn/</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Expert Insulation</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>info@larsonkeeney.com</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>608-222-9919</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Rochester MN</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>100</v>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>roofing contractor Rochester MN</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 13:19 UTC (cycle 20)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L74"/>
+  <dimension ref="A1:L75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4778,6 +4778,66 @@
         </is>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Barnett Plumbing</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>barnettplumber.com</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>https://barnettplumber.com/</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>At Barnett</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>info@barnettplumbing.com</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>678-437-1234</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Marietta GA</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>100</v>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>plumbing company Marietta GA</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 13:20 UTC (cycle 21)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L75"/>
+  <dimension ref="A1:L76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4838,6 +4838,66 @@
         </is>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Roofing Company in Broken Arrow, OK | Roof Works</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>brokenarrowroofworks.com</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>https://brokenarrowroofworks.com/</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Questions Broken</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>hello@brokenarrowroofworks.com</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>(918) 359-2694</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Broken Arrow OK</t>
+        </is>
+      </c>
+      <c r="I76" t="n">
+        <v>100</v>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>roof repair company Broken Arrow OK</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 13:23 UTC (cycle 23)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L76"/>
+  <dimension ref="A1:L79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4898,6 +4898,186 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Roof Replacement &amp; Repair in Grand Prairie, TX | Gibco Roofing</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>gibcoroofingandremodeling.com</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>https://gibcoroofingandremodeling.com/service-areas/grand-prairie</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Gibco Roofing</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>carlos@gibcoroofingandremodeling.com</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>(972) 352-3479</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Grand Prairie TX</t>
+        </is>
+      </c>
+      <c r="I77" t="n">
+        <v>100</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>roof repair company Grand Prairie TX</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Clean Heat Rhode Island</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>cleanheatri.com</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>https://cleanheatri.com/resources/find-an-installer/</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Toggle Navigation</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>cleanheatri@abodeenergy.com</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>(401) 300-1880</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Providence RI</t>
+        </is>
+      </c>
+      <c r="I78" t="n">
+        <v>98</v>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>heat pump installation Providence RI</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Envr Air</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>envrair.com</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>https://envrair.com/</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Jesse Mastro</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>hello@envrair.com</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>(855) 791-3040</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Providence RI</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
+        <v>96</v>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>heat pump installation Providence RI</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 13:25 UTC (cycle 24)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L79"/>
+  <dimension ref="A1:L80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5078,6 +5078,66 @@
         </is>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Plumber in New Braunfels, TX | Plunger Pros</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>plungerprostx.com</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>https://plungerprostx.com/</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Plunger Pros</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>office@plungerprostx.com</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>(830) 356-2141</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
+        <v>90</v>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>plumber New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 13:28 UTC (cycle 26)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L80"/>
+  <dimension ref="A1:L81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5138,6 +5138,66 @@
         </is>
       </c>
     </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Cool Fox Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>coolfoxheating.com</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>https://coolfoxheating.com/heat-pump-installation-in-bellevue-wa/</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Built On</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>info@coolfoxheating.com</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>253) 368-3068</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Bellevue WA</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>100</v>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>heat pump installation Bellevue WA</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 13:37 UTC (cycle 32)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L81"/>
+  <dimension ref="A1:L82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5198,6 +5198,62 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>BETLEM RESIDENTIAL Heating &amp; Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>betlem.com</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>https://www.betlem.com/</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>residential@betlem.com</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>585.271.4328</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Rochester NY</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
+        <v>66</v>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>heating and cooling company Rochester NY</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 13:40 UTC (cycle 34)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L82"/>
+  <dimension ref="A1:L83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5219,7 +5219,6 @@
           <t>https://www.betlem.com/</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr">
         <is>
           <t>residential@betlem.com</t>
@@ -5249,6 +5248,66 @@
         </is>
       </c>
       <c r="L82" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Roof Monsters</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>roofmonsters.co</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>https://roofmonsters.co/about-us/locations-we-serve/roofing-company-clearwater-florida/</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>View Dunedin</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>info@roofmonsters.co</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>(727) 439-3869</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Clearwater FL</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
+        <v>100</v>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>roof repair company Clearwater FL</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 13:41 UTC (cycle 35)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L83"/>
+  <dimension ref="A1:L84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5313,6 +5313,62 @@
         </is>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Water Heater Repair Stockton | 24hr Water Heater Replacement Services | Free Plu</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>waterheaterrepairstockton.com</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>https://waterheaterrepairstockton.com/</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>stocktonwaterheaters@gmail.com</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>(209) 353-9777</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Stockton CA</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>100</v>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>water heater repair Stockton CA</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 13:44 UTC (cycle 37)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L84"/>
+  <dimension ref="A1:L85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5334,7 +5334,6 @@
           <t>https://waterheaterrepairstockton.com/</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr">
         <is>
           <t>stocktonwaterheaters@gmail.com</t>
@@ -5364,6 +5363,62 @@
         </is>
       </c>
       <c r="L84" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>24/7 Air Solution</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>247airsolution.com</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>https://247airsolution.com/locations/coral-springs</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>247airsolution@gmail.com</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>(855) 417-8866</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Coral Springs FL</t>
+        </is>
+      </c>
+      <c r="I85" t="n">
+        <v>100</v>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>air conditioning repair Coral Springs FL</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 13:46 UTC (cycle 38)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L85"/>
+  <dimension ref="A1:L86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5389,7 +5389,6 @@
           <t>https://247airsolution.com/locations/coral-springs</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr">
         <is>
           <t>247airsolution@gmail.com</t>
@@ -5419,6 +5418,66 @@
         </is>
       </c>
       <c r="L85" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Curry Plumbing</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>curryplumbing.com</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>https://curryplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Scott Curry</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>curryco@curryplumbing.com</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>863.644.0061</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Lakeland FL</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>90</v>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>plumbing company Lakeland FL</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 13:56 UTC (cycle 45)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L86"/>
+  <dimension ref="A1:L87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5483,6 +5483,66 @@
         </is>
       </c>
     </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Roof City Inc</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>roofcityprofessionals.com</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>https://roofcityprofessionals.com/roof-repair-in-elk-grove</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Hugo Rodriguez</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>info@roofcityprofessionals.com</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>916-943-4374</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Elk Grove CA</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>90</v>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>roof repair company Elk Grove CA</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 13:59 UTC (cycle 47)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L87"/>
+  <dimension ref="A1:L88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5543,6 +5543,62 @@
         </is>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Show Me Metal Roofing</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>showmemetalroofing.com</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>https://showmemetalroofing.com/locations/columbia/</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Show Me</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>compassleadgroup@gmail.com</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr"/>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Columbia MO</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>84</v>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Columbia MO</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 14:02 UTC (cycle 49)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L88"/>
+  <dimension ref="A1:L90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5574,7 +5574,6 @@
           <t>compassleadgroup@gmail.com</t>
         </is>
       </c>
-      <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
           <t>Columbia MO</t>
@@ -5594,6 +5593,126 @@
         </is>
       </c>
       <c r="L88" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Professional Roofing &amp; Storm Restoration | Veteran's Choice Contracting | Davenp</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>veteranschoicecontracting.com</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>https://www.veteranschoicecontracting.com/</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Rock Isl</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>shaine@veteranschoicecontracting.com</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>(563)-424-1005</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Davenport IA</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>100</v>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>roofing contractor Davenport IA</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Roofing Services | Sieren Roofing Services | Davenport, IA</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>sierenroofing.com</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>https://www.sierenroofing.com/</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Quad Cities</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>sierenroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>(563) 549-0279</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Davenport IA</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>98</v>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>roofing contractor Davenport IA</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 14:14 UTC (cycle 57)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L90"/>
+  <dimension ref="A1:L91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5718,6 +5718,62 @@
         </is>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>1231893.us8.myftpupload.com Managed WordPress Site</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>nelaroofing.com</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>https://nelaroofing.com/locations/jackson-mississippi/</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>sales@nelaroofing.com</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>318-737-1999</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Jackson MS</t>
+        </is>
+      </c>
+      <c r="I91" t="n">
+        <v>82</v>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>roofer Jackson MS</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 14:17 UTC (cycle 59)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L91"/>
+  <dimension ref="A1:L92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5739,7 +5739,6 @@
           <t>https://nelaroofing.com/locations/jackson-mississippi/</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
           <t>sales@nelaroofing.com</t>
@@ -5769,6 +5768,62 @@
         </is>
       </c>
       <c r="L91" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>DeepSouth AC - Dev Site</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>deepsouthac.com</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>https://deepsouthac.com/</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>info@deepsouthac.com</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>(337) 417-8714</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Lafayette LA</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
+        <v>90</v>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>heating and cooling company Lafayette LA</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 14:20 UTC (cycle 61)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L92"/>
+  <dimension ref="A1:L93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5794,7 +5794,6 @@
           <t>https://deepsouthac.com/</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
           <t>info@deepsouthac.com</t>
@@ -5824,6 +5823,66 @@
         </is>
       </c>
       <c r="L92" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Driftwood Plumbing and Heating</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>driftwoodplumbing.com</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>https://driftwoodplumbing.com/renton-wa</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Driftwood Plumbing</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>info@driftwoodplumbing.com</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>(253) 693-8693</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Renton WA</t>
+        </is>
+      </c>
+      <c r="I93" t="n">
+        <v>90</v>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>plumbing company Renton WA</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 14:21 UTC (cycle 62)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L93"/>
+  <dimension ref="A1:L94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5888,6 +5888,66 @@
         </is>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Roof Replacement | Roof Installation | Santa Fe, NM</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>abcroofingspecialistlosalamos.com</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>https://www.abcroofingspecialistlosalamos.com/roof-replacement</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Santa Fe</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>silviano@abcroofspecialists.com</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>(505) 594-1506</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Santa Fe NM</t>
+        </is>
+      </c>
+      <c r="I94" t="n">
+        <v>100</v>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>roof replacement Santa Fe NM</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 14:33 UTC (cycle 70)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L94"/>
+  <dimension ref="A1:L95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5948,6 +5948,66 @@
         </is>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>St. Pierre Plumbing &amp; Drain Cleaning</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>stpierreplumbing.com</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>https://stpierreplumbing.com/areas-we-serve/concord-nh/</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Pierre Jr</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>info@stpierreplumbing.com</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>(603) 560-2416</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Concord NH</t>
+        </is>
+      </c>
+      <c r="I95" t="n">
+        <v>100</v>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>plumbing company Concord NH</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 14:48 UTC (cycle 80)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L95"/>
+  <dimension ref="A1:L96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6008,6 +6008,62 @@
         </is>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>TBT HVAC</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>tbthvac.com</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>https://tbthvac.com/service/ac-installation-in-nashville/</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>tbthvac4@gmail.com</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>615.708.8383</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Nashville TN</t>
+        </is>
+      </c>
+      <c r="I96" t="n">
+        <v>100</v>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>AC installation Nashville TN</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 14:54 UTC (cycle 84)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L96"/>
+  <dimension ref="A1:L97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6029,7 +6029,6 @@
           <t>https://tbthvac.com/service/ac-installation-in-nashville/</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr">
         <is>
           <t>tbthvac4@gmail.com</t>
@@ -6059,6 +6058,62 @@
         </is>
       </c>
       <c r="L96" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Aylwin Construction</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>aylwinconstruction.com</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>https://aylwinconstruction.com/</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>info@roofpdx.com</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>(503) 998-7663</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Hillsboro OR</t>
+        </is>
+      </c>
+      <c r="I97" t="n">
+        <v>90</v>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>roof replacement Hillsboro OR</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 15:00 UTC (cycle 88)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L97"/>
+  <dimension ref="A1:L98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6084,7 +6084,6 @@
           <t>https://aylwinconstruction.com/</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
         <is>
           <t>info@roofpdx.com</t>
@@ -6114,6 +6113,66 @@
         </is>
       </c>
       <c r="L97" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Big Sky Roofing Inc.</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>bigskyroofingfl.com</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>https://bigskyroofingfl.com/ocala-fl/</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Altamonte Springs</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>info@bigskyroofingfl.com</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>(352) 603-2458</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Ocala FL</t>
+        </is>
+      </c>
+      <c r="I98" t="n">
+        <v>90</v>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>residential roofing company Ocala FL</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 15:04 UTC (cycle 91)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L98"/>
+  <dimension ref="A1:L99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6178,6 +6178,66 @@
         </is>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Local Roofing Jersey City</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>localroofingjerseycity.com</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>https://localroofingjerseycity.com/</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Roofing Jersey</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>hello@plumber.com</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>201-942-1832</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Jersey City NJ</t>
+        </is>
+      </c>
+      <c r="I99" t="n">
+        <v>100</v>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>roofing contractor Jersey City NJ</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 15:10 UTC (cycle 95)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L99"/>
+  <dimension ref="A1:L100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6238,6 +6238,62 @@
         </is>
       </c>
     </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Sewer Line Repair in Bakersfield, CA</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>plumbsd.com</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>https://plumbsd.com/services/sewer-line/bakersfield/</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>contact@plumbsd.com</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>(833) 546-3641</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Bakersfield CA</t>
+        </is>
+      </c>
+      <c r="I100" t="n">
+        <v>90</v>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>sewer repair Bakersfield CA</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 15:19 UTC (cycle 101)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L100"/>
+  <dimension ref="A1:L101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6259,7 +6259,6 @@
           <t>https://plumbsd.com/services/sewer-line/bakersfield/</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr">
         <is>
           <t>contact@plumbsd.com</t>
@@ -6289,6 +6288,66 @@
         </is>
       </c>
       <c r="L100" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Ehrhardt Brothers Quality Plumbing, Inc.</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>columbiaplumber.com</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>https://columbiaplumber.com/</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Virtual Estimate</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>office@columbiaplumber.net</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>(410) 997-8414</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Columbia MD</t>
+        </is>
+      </c>
+      <c r="I101" t="n">
+        <v>90</v>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>plumbing company Columbia MD</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 15:25 UTC (cycle 105)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L101"/>
+  <dimension ref="A1:L102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6353,6 +6353,62 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Red Letter Roofing</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>redletterroofing.com</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>https://redletterroofing.com/durham-roofing/</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>info@redletterroofing.com</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>919-977-5318</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Durham NC</t>
+        </is>
+      </c>
+      <c r="I102" t="n">
+        <v>100</v>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>roofer Durham NC</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 15:32 UTC (cycle 110)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L102"/>
+  <dimension ref="A1:L103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6374,7 +6374,6 @@
           <t>https://redletterroofing.com/durham-roofing/</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
           <t>info@redletterroofing.com</t>
@@ -6404,6 +6403,66 @@
         </is>
       </c>
       <c r="L102" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>HVAC Repair Aurora</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>hvacrepairaurora.com</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>https://hvacrepairaurora.com/</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>West Chicago</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>faridahmad1050@gmail.com</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>(630) 467-6249</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Aurora IL</t>
+        </is>
+      </c>
+      <c r="I103" t="n">
+        <v>94</v>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>air conditioning repair Aurora IL</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 15:34 UTC (cycle 111)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L103"/>
+  <dimension ref="A1:L104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6468,6 +6468,66 @@
         </is>
       </c>
     </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Native Roofing + Construction</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>nativeroofingok.com</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>https://www.nativeroofingok.com/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Team Blake</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>info@nativeroofingok.com</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>(918) 552-0655</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Tulsa OK</t>
+        </is>
+      </c>
+      <c r="I104" t="n">
+        <v>96</v>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Tulsa OK</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 15:35 UTC (cycle 112)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L104"/>
+  <dimension ref="A1:L106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6528,6 +6528,118 @@
         </is>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Expert Metal Roofing in Tacoma, WA | South Sound Roofing LLC</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>southsoundroofingllc.com</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>https://southsoundroofingllc.com/geo/metal-roofing-tacoma-wa</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>merinolorenzo756@gmail.com</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>360-771-7637</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Tacoma WA</t>
+        </is>
+      </c>
+      <c r="I105" t="n">
+        <v>94</v>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Tacoma WA</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Metal Roofing in Tacoma, WA | Prestige Prime Construction LLC</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>prestigeprimeconstructionllc.com</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>https://prestigeprimeconstructionllc.com/services/metal-roofing-in-tacoma-wa</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>gat26cami@icloud.com</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>360-523-0620</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Tacoma WA</t>
+        </is>
+      </c>
+      <c r="I106" t="n">
+        <v>84</v>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Tacoma WA</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 15:47 UTC (cycle 120)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L106"/>
+  <dimension ref="A1:L107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6549,7 +6549,6 @@
           <t>https://southsoundroofingllc.com/geo/metal-roofing-tacoma-wa</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
         <is>
           <t>merinolorenzo756@gmail.com</t>
@@ -6605,7 +6604,6 @@
           <t>https://prestigeprimeconstructionllc.com/services/metal-roofing-in-tacoma-wa</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
         <is>
           <t>gat26cami@icloud.com</t>
@@ -6635,6 +6633,66 @@
         </is>
       </c>
       <c r="L106" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>ClearPath Plumbing and Drain Cleaning Solutions</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>cpplumbingdrain.com</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>https://www.cpplumbingdrain.com/services/sewer-line-inspection-repair/</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>With Dedication</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>cpplumbingdrainsolutions@gmail.com</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>(209) 918-8500</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Modesto CA</t>
+        </is>
+      </c>
+      <c r="I107" t="n">
+        <v>100</v>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>sewer repair Modesto CA</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 15:50 UTC (cycle 122)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L107"/>
+  <dimension ref="A1:L108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6698,6 +6698,62 @@
         </is>
       </c>
     </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Readyman Pros Heatin</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>readymanheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>https://www.readymanheatingandcooling.com/</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>info@mysite.com</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>(541) 991-5107</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Bend OR</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
+        <v>88</v>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>heating and cooling company Bend OR</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 15:55 UTC (cycle 125)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L108"/>
+  <dimension ref="A1:L109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6719,7 +6719,6 @@
           <t>https://www.readymanheatingandcooling.com/</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr">
         <is>
           <t>info@mysite.com</t>
@@ -6749,6 +6748,62 @@
         </is>
       </c>
       <c r="L108" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Magic Metals Manufacturing</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>magicmetalsinc.com</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>https://magicmetalsinc.com/</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>sales@magicmetalsinc.com</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>907.746.7800</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Anchorage AK</t>
+        </is>
+      </c>
+      <c r="I109" t="n">
+        <v>82</v>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Anchorage AK</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 15:59 UTC (cycle 128)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L109"/>
+  <dimension ref="A1:L110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6774,7 +6774,6 @@
           <t>https://magicmetalsinc.com/</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr">
         <is>
           <t>sales@magicmetalsinc.com</t>
@@ -6804,6 +6803,62 @@
         </is>
       </c>
       <c r="L109" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Sewer Line Repair in Alpharetta, GA</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>alpharetta-ga.kbuenoplumbing.com</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>https://alpharetta-ga.kbuenoplumbing.com/sewer-line-repair/</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>contact@kbuenoplumbing.com</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>(888) 576-6192</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Alpharetta GA</t>
+        </is>
+      </c>
+      <c r="I110" t="n">
+        <v>90</v>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>sewer repair Alpharetta GA</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 16:21 UTC (cycle 143)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L110"/>
+  <dimension ref="A1:L111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6829,7 +6829,6 @@
           <t>https://alpharetta-ga.kbuenoplumbing.com/sewer-line-repair/</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr">
         <is>
           <t>contact@kbuenoplumbing.com</t>
@@ -6859,6 +6858,66 @@
         </is>
       </c>
       <c r="L110" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Hialeah Metal Roof</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>hialeahmetalroof.com</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>https://hialeahmetalroof.com/</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Questions Hialeah</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>info@hialeahmetalroof.com</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>786-460-2101</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Hialeah FL</t>
+        </is>
+      </c>
+      <c r="I111" t="n">
+        <v>90</v>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Hialeah FL</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 16:46 UTC (cycle 160)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L111"/>
+  <dimension ref="A1:L112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6923,6 +6923,66 @@
         </is>
       </c>
     </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>GreenFlow Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>greenflowhvac.com</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>https://greenflowhvac.com/hvac-services-federal-way-wa/</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>What Makes</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>njoslin@greenflowhvac.com</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>253-370-8641</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Federal Way WA</t>
+        </is>
+      </c>
+      <c r="I112" t="n">
+        <v>90</v>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>heat pump installation Federal Way WA</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 17:04 UTC (cycle 172)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L112"/>
+  <dimension ref="A1:L113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6983,6 +6983,66 @@
         </is>
       </c>
     </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Professional Choice Plumbing</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>professionalchoicefl.com</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>https://www.professionalchoicefl.com/</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Professional Choice</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>info@professionalchoicefl.com</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>(352) 778-1002</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Ocala FL</t>
+        </is>
+      </c>
+      <c r="I113" t="n">
+        <v>90</v>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>plumbing company Ocala FL</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 17:14 UTC (cycle 179)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L113"/>
+  <dimension ref="A1:L114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7043,6 +7043,66 @@
         </is>
       </c>
     </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Air-Right</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>airrightac.com</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>https://airrightac.com/heat-pump/heat-pump-installation-replacement-north-las-vegas-nv</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Service Rapid</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>info@airrightac.com</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>(702) 979-1519</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>North Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="I114" t="n">
+        <v>90</v>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>heat pump installation North Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 17:22 UTC (cycle 184)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L114"/>
+  <dimension ref="A1:L115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7103,6 +7103,66 @@
         </is>
       </c>
     </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Rock Solid Exteriors</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>rocksolidexteriors.com</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>https://rocksolidexteriors.com/roofing/sterling-heights-mi/</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Rock Solid</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>hello@rocksolidexteriors.com</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>(844) 757-6543</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Sterling Heights MI</t>
+        </is>
+      </c>
+      <c r="I115" t="n">
+        <v>100</v>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>residential roofing company Sterling Heights MI</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 17:27 UTC (cycle 188)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L115"/>
+  <dimension ref="A1:L116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7163,6 +7163,66 @@
         </is>
       </c>
     </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Pro Bid LLC</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>probidconstruction.com</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>https://probidconstruction.com/sewer-drain-services/sewer-line-repair/</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>At Pro</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>info@probidspringfield.com</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>217.971.7555</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Springfield IL</t>
+        </is>
+      </c>
+      <c r="I116" t="n">
+        <v>100</v>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>sewer repair Springfield IL</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 17:32 UTC (cycle 191)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L116"/>
+  <dimension ref="A1:L117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7223,6 +7223,62 @@
         </is>
       </c>
     </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Ethical Plumbing</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>ethicalplumbing.com</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>https://ethicalplumbing.com/greenville-sc/emergency-plumber/</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>help@ethicalplumbing.net</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>864-438-0525</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Greenville SC</t>
+        </is>
+      </c>
+      <c r="I117" t="n">
+        <v>100</v>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>emergency plumber Greenville SC</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 17:33 UTC (cycle 192)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L117"/>
+  <dimension ref="A1:L118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7244,7 +7244,6 @@
           <t>https://ethicalplumbing.com/greenville-sc/emergency-plumber/</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr">
         <is>
           <t>help@ethicalplumbing.net</t>
@@ -7274,6 +7273,66 @@
         </is>
       </c>
       <c r="L117" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Zero Homes</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>zerohomes.com</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>https://www.zerohomes.com/locations/arvada-co/heat-pump-installer</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Tristate Rural</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>hello@zerohomes.com</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>(303) 848-8606</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Arvada CO</t>
+        </is>
+      </c>
+      <c r="I118" t="n">
+        <v>80</v>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>heat pump installation Arvada CO</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 17:44 UTC (cycle 199)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L118"/>
+  <dimension ref="A1:L119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7338,6 +7338,66 @@
         </is>
       </c>
     </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Pratt Plumbing</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>prattplumbing.net</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>https://prattplumbing.net/amarillos-best-plumbing-services/amarillo-drain-cleaning/</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>John Esler</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>info@prattplumbing.net</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>806.373.7866</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Amarillo TX</t>
+        </is>
+      </c>
+      <c r="I119" t="n">
+        <v>100</v>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>drain cleaning service Amarillo TX</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 17:50 UTC (cycle 203)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L119"/>
+  <dimension ref="A1:L121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7398,6 +7398,126 @@
         </is>
       </c>
     </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Metal Roofing Waterbury</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>cmroofingco.com</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>https://cmroofingco.com/areas-of-service/waterbury-metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Commercial Roofing</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>info@cmroofingco.com</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>(860) 758-7708</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Waterbury CT</t>
+        </is>
+      </c>
+      <c r="I120" t="n">
+        <v>100</v>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Waterbury CT</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Gold Seal</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>goldsealplumbing.com</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>https://www.goldsealplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Richard Dixon</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>amandad@goldsealplumbing.com</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>(509) 535-5946</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Spokane WA</t>
+        </is>
+      </c>
+      <c r="I121" t="n">
+        <v>90</v>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>plumbing company Spokane WA</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 19:09 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L121"/>
+  <dimension ref="A1:L122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7518,6 +7518,66 @@
         </is>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Premier Heating and Cooling | Serving St. Louis and St. Charles Missouri</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>premierheatingcooling.net</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>https://premierheatingcooling.net/</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>What Does</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>service@premierheatingcooling.net</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>(636) 916-1122</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>St Charles MO</t>
+        </is>
+      </c>
+      <c r="I122" t="n">
+        <v>100</v>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>heating and cooling company St Charles MO</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 19:11 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L122"/>
+  <dimension ref="A1:L123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7578,6 +7578,58 @@
         </is>
       </c>
     </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Roof Repair &amp; Replacement</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>lanceroofing.com</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>https://lanceroofing.com/services/roofing/</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>jan@lanceroofing.com</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr"/>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Dayton OH</t>
+        </is>
+      </c>
+      <c r="I123" t="n">
+        <v>86</v>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Dayton OH</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 19:14 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L123"/>
+  <dimension ref="A1:L125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7599,13 +7599,11 @@
           <t>https://lanceroofing.com/services/roofing/</t>
         </is>
       </c>
-      <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr">
         <is>
           <t>jan@lanceroofing.com</t>
         </is>
       </c>
-      <c r="G123" t="inlineStr"/>
       <c r="H123" t="inlineStr">
         <is>
           <t>Dayton OH</t>
@@ -7625,6 +7623,126 @@
         </is>
       </c>
       <c r="L123" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Houston Roof Repair</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>houstonroofrepair.com</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>https://houstonroofrepair.com/the-woodlands-roofing-company/</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>On Over</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>info@houstonroofrepair.com</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>832-271-4991</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>The Woodlands TX</t>
+        </is>
+      </c>
+      <c r="I124" t="n">
+        <v>100</v>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>roof repair company The Woodlands TX</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>John's Plumbing &amp; Heating NY</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>johnsplumbingny.com</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>https://johnsplumbingny.com/</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Heating Service</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>info@johnsplumbingny.com</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>718-295-4263</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Bronx NY</t>
+        </is>
+      </c>
+      <c r="I125" t="n">
+        <v>100</v>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>plumbing company Bronx NY</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 19:22 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L125"/>
+  <dimension ref="A1:L126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7748,6 +7748,62 @@
         </is>
       </c>
     </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Residential Roofing in Queens, NY | Wetherall Roofing</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>wetherallroofingandcontracting.com</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>https://www.wetherallroofingandcontracting.com/residential-roofing-in-queens--ny</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr"/>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>info@wetherallroofingandcontracting.com</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>(718) 894-7011</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Queens NY</t>
+        </is>
+      </c>
+      <c r="I126" t="n">
+        <v>90</v>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>residential roofing company Queens NY</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 19:24 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L126"/>
+  <dimension ref="A1:L127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7769,7 +7769,6 @@
           <t>https://www.wetherallroofingandcontracting.com/residential-roofing-in-queens--ny</t>
         </is>
       </c>
-      <c r="E126" t="inlineStr"/>
       <c r="F126" t="inlineStr">
         <is>
           <t>info@wetherallroofingandcontracting.com</t>
@@ -7799,6 +7798,66 @@
         </is>
       </c>
       <c r="L126" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Residential Roofing | Fredericksburg, VA | John Mills Jr</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>johnmillsroofing.com</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>https://www.johnmillsroofing.com/home-roofing-services</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>John Mills</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>johnmillsroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>(540) 582-7499</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>Fredericksburg VA</t>
+        </is>
+      </c>
+      <c r="I127" t="n">
+        <v>90</v>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>residential roofing company Fredericksburg VA</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 19:26 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L127"/>
+  <dimension ref="A1:L128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7863,6 +7863,66 @@
         </is>
       </c>
     </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Marietta HVAC Pros</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>mariettahvacpros.com</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>https://mariettahvacpros.com/</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Reviews What</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>handyheroesinc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>470-847-9076</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>Marietta GA</t>
+        </is>
+      </c>
+      <c r="I128" t="n">
+        <v>70</v>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>HVAC contractor Marietta GA</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 19:28 UTC (cycle 15)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L128"/>
+  <dimension ref="A1:L129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7923,6 +7923,62 @@
         </is>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Plumbing Company Florida</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>tallahassee.plumbingcompanyflorida.com</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>https://tallahassee.plumbingcompanyflorida.com/</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr"/>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>dispatch@plumbingcompanyflorida.com</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>407-598-8903</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>Tallahassee FL</t>
+        </is>
+      </c>
+      <c r="I129" t="n">
+        <v>100</v>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>emergency plumber Tallahassee FL</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 19:31 UTC (cycle 17)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L129"/>
+  <dimension ref="A1:L130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7944,7 +7944,6 @@
           <t>https://tallahassee.plumbingcompanyflorida.com/</t>
         </is>
       </c>
-      <c r="E129" t="inlineStr"/>
       <c r="F129" t="inlineStr">
         <is>
           <t>dispatch@plumbingcompanyflorida.com</t>
@@ -7974,6 +7973,66 @@
         </is>
       </c>
       <c r="L129" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Mak - El Paso Roofing &amp; Construction</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>elpasoroofings.com</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>https://elpasoroofings.com/top-10-residential-roofing-contractors-in-el-paso/</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>El Paso</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>makconstruction.us@gmail.com</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>915-691-0532</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>El Paso TX</t>
+        </is>
+      </c>
+      <c r="I130" t="n">
+        <v>90</v>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>residential roofing company El Paso TX</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 19:34 UTC (cycle 19)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L130"/>
+  <dimension ref="A1:L131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8038,6 +8038,66 @@
         </is>
       </c>
     </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Brownsville Roofing Services</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>arrowroofingtx.com</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>https://www.arrowroofingtx.com/locations/brownsville</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Arrow Roofing</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>info@arrowroofingtx.com</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>(956) 374-7447</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Brownsville TX</t>
+        </is>
+      </c>
+      <c r="I131" t="n">
+        <v>100</v>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Brownsville TX</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 19:36 UTC (cycle 20)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L131"/>
+  <dimension ref="A1:L133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8098,6 +8098,118 @@
         </is>
       </c>
     </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Roofing Contractor Riverside CA | Roof Repair &amp; Replacement | Roofing and More</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>roofingandmorellc.com</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>https://www.roofingandmorellc.com/</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr"/>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>hello@roofingandmorellc.com</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>(951) 720-1209</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>Riverside CA</t>
+        </is>
+      </c>
+      <c r="I132" t="n">
+        <v>90</v>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>roofing contractor Riverside CA</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>American Roofing</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>americanroofingltd.com</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>https://www.americanroofingltd.com/residential-home</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr"/>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>treyh@americanroofingltd.com</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>(281) 367-7666</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>The Woodlands TX</t>
+        </is>
+      </c>
+      <c r="I133" t="n">
+        <v>90</v>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>residential roofing company The Woodlands TX</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 19:42 UTC (cycle 24)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L133"/>
+  <dimension ref="A1:L135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8119,7 +8119,6 @@
           <t>https://www.roofingandmorellc.com/</t>
         </is>
       </c>
-      <c r="E132" t="inlineStr"/>
       <c r="F132" t="inlineStr">
         <is>
           <t>hello@roofingandmorellc.com</t>
@@ -8175,7 +8174,6 @@
           <t>https://www.americanroofingltd.com/residential-home</t>
         </is>
       </c>
-      <c r="E133" t="inlineStr"/>
       <c r="F133" t="inlineStr">
         <is>
           <t>treyh@americanroofingltd.com</t>
@@ -8205,6 +8203,122 @@
         </is>
       </c>
       <c r="L133" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Aire Serv of Vancouver</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>aireservvancouver.com</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>https://aireservvancouver.com/areas-we-service/vancouver-washington/</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr"/>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>info@aireservvancouver.com</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>(360) 524-3952</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>Vancouver WA</t>
+        </is>
+      </c>
+      <c r="I134" t="n">
+        <v>100</v>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>air conditioning repair Vancouver WA</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Beemans Heating &amp; Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>beemansheatingandairconditioning.com</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>https://www.beemansheatingandairconditioning.com/</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Learn More</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>beemansheating8@gmail.com</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>(360) 762-2733</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>Vancouver WA</t>
+        </is>
+      </c>
+      <c r="I135" t="n">
+        <v>90</v>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>air conditioning repair Vancouver WA</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 19:43 UTC (cycle 25)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L135"/>
+  <dimension ref="A1:L136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8229,7 +8229,6 @@
           <t>https://aireservvancouver.com/areas-we-service/vancouver-washington/</t>
         </is>
       </c>
-      <c r="E134" t="inlineStr"/>
       <c r="F134" t="inlineStr">
         <is>
           <t>info@aireservvancouver.com</t>
@@ -8319,6 +8318,66 @@
         </is>
       </c>
       <c r="L135" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>HVAC Contractor | Aurora, Colorado</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>nitroheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>https://www.nitroheatingandcooling.com/</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>To Nitro</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>services@nitroheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>720-415-3336</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>Aurora CO</t>
+        </is>
+      </c>
+      <c r="I136" t="n">
+        <v>90</v>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>HVAC contractor Aurora CO</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 19:47 UTC (cycle 28)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L136"/>
+  <dimension ref="A1:L138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8383,6 +8383,122 @@
         </is>
       </c>
     </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>OKC Roofing Services</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>okcroofingservices.com</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>https://okcroofingservices.com/locations/norman/</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Roofing Services</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>info@okcroofingservices.com</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>(405) 555-0199</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>Norman OK</t>
+        </is>
+      </c>
+      <c r="I137" t="n">
+        <v>100</v>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>roof replacement Norman OK</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Halo Roofing and Construction | Roof Replacements Norman OK</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>haloroofs.com</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>https://www.haloroofs.com/</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr"/>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>sales@haloroofs.com</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>405-317-7405</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>Norman OK</t>
+        </is>
+      </c>
+      <c r="I138" t="n">
+        <v>96</v>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>roof replacement Norman OK</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 20:02 UTC (cycle 38)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L138"/>
+  <dimension ref="A1:L139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8464,7 +8464,6 @@
           <t>https://www.haloroofs.com/</t>
         </is>
       </c>
-      <c r="E138" t="inlineStr"/>
       <c r="F138" t="inlineStr">
         <is>
           <t>sales@haloroofs.com</t>
@@ -8494,6 +8493,62 @@
         </is>
       </c>
       <c r="L138" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Elite Florida Roofers</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>elitefloridaroofers.com</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>https://elitefloridaroofers.com/west-palm-beach-roofing-company/</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr"/>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>info@ndcreditrepair.com</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>245 253 2125</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>West Palm Beach FL</t>
+        </is>
+      </c>
+      <c r="I139" t="n">
+        <v>100</v>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>residential roofing company West Palm Beach FL</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 20:06 UTC (cycle 41)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L139"/>
+  <dimension ref="A1:L140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8519,7 +8519,6 @@
           <t>https://elitefloridaroofers.com/west-palm-beach-roofing-company/</t>
         </is>
       </c>
-      <c r="E139" t="inlineStr"/>
       <c r="F139" t="inlineStr">
         <is>
           <t>info@ndcreditrepair.com</t>
@@ -8549,6 +8548,62 @@
         </is>
       </c>
       <c r="L139" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Ken-Z Roofing</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>kenzroofing.com</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>https://www.kenzroofing.com/</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr"/>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>kenzroof@aol.com</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>815-395-8244</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>Rockford IL</t>
+        </is>
+      </c>
+      <c r="I140" t="n">
+        <v>96</v>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>roofer Rockford IL</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 20:18 UTC (cycle 49)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L140"/>
+  <dimension ref="A1:L141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8574,7 +8574,6 @@
           <t>https://www.kenzroofing.com/</t>
         </is>
       </c>
-      <c r="E140" t="inlineStr"/>
       <c r="F140" t="inlineStr">
         <is>
           <t>kenzroof@aol.com</t>
@@ -8604,6 +8603,66 @@
         </is>
       </c>
       <c r="L140" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Mountain Man Plumbing</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>mtnmanplumbing.com</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>https://mtnmanplumbing.com/west-jordan-plumber/</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Tyler Nerdin</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>tyler@mtnmanplumbing.com</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>(385) 766-8935</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>West Jordan UT</t>
+        </is>
+      </c>
+      <c r="I141" t="n">
+        <v>90</v>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>plumber West Jordan UT</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 20:22 UTC (cycle 52)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L141"/>
+  <dimension ref="A1:L142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8668,6 +8668,66 @@
         </is>
       </c>
     </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Irving Roofing Company</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>lonestarroofers.com</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>https://lonestarroofers.com/texas/irving-roofing</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Fort Worth</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>sales@lonestarroofers.com</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>972-816-8967</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>Irving TX</t>
+        </is>
+      </c>
+      <c r="I142" t="n">
+        <v>100</v>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>residential roofing company Irving TX</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 20:34 UTC (cycle 60)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L142"/>
+  <dimension ref="A1:L143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8728,6 +8728,66 @@
         </is>
       </c>
     </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>South Placer Heating and Air</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>placerheatingandair.com</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>https://www.placerheatingandair.com/areas-served/stockton/</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Northern California</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>scott@southplacerha.com</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>(916) 246-2089</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Stockton CA</t>
+        </is>
+      </c>
+      <c r="I143" t="n">
+        <v>100</v>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>heat pump installation Stockton CA</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 20:41 UTC (cycle 65)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L143"/>
+  <dimension ref="A1:L144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8788,6 +8788,62 @@
         </is>
       </c>
     </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>911 Plumbing Conroe</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>911plumbingconroe.com</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>https://911plumbingconroe.com/sewer-repair.html</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr"/>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>service@911plumbingconroe.com</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>(936) 344-3134</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>Conroe TX</t>
+        </is>
+      </c>
+      <c r="I144" t="n">
+        <v>100</v>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>sewer repair Conroe TX</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 20:52 UTC (cycle 72)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L144"/>
+  <dimension ref="A1:L146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8809,7 +8809,6 @@
           <t>https://911plumbingconroe.com/sewer-repair.html</t>
         </is>
       </c>
-      <c r="E144" t="inlineStr"/>
       <c r="F144" t="inlineStr">
         <is>
           <t>service@911plumbingconroe.com</t>
@@ -8839,6 +8838,126 @@
         </is>
       </c>
       <c r="L144" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>HVAC Company New Jersey</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>heat-pump-installation-trenton.aeshvacnj.com</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>https://heat-pump-installation-trenton.aeshvacnj.com/</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Call Us</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>example@mail.com</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>(888) 978-1291</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>Trenton NJ</t>
+        </is>
+      </c>
+      <c r="I145" t="n">
+        <v>100</v>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>heat pump installation Trenton NJ</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Sines and Sons Heating and Cooling | Arnold, MD</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>sinesandsons.com</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>https://sinesandsons.com/annapolis-md/</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Why Homeowners</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>sinesacace2020@gmail.com</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>(410) 267-0260</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>Annapolis MD</t>
+        </is>
+      </c>
+      <c r="I146" t="n">
+        <v>80</v>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>heating and cooling company Annapolis MD</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 20:53 UTC (cycle 73)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L146"/>
+  <dimension ref="A1:L147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8963,6 +8963,62 @@
         </is>
       </c>
     </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>King Arthur Plumbing - NJ Plumber Heating Air Conditioning New Jersey HVAC Sewer</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>kingarthurplumbing.com</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>https://kingarthurplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr"/>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>info@kingarthurplumbing.com</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>(732) 734-1350</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>Woodbridge NJ</t>
+        </is>
+      </c>
+      <c r="I147" t="n">
+        <v>100</v>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>plumbing company Woodbridge NJ</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 20:54 UTC (cycle 74)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L147"/>
+  <dimension ref="A1:L148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8984,7 +8984,6 @@
           <t>https://kingarthurplumbing.com/</t>
         </is>
       </c>
-      <c r="E147" t="inlineStr"/>
       <c r="F147" t="inlineStr">
         <is>
           <t>info@kingarthurplumbing.com</t>
@@ -9014,6 +9013,62 @@
         </is>
       </c>
       <c r="L147" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Craftsmen Home Improvements</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>craftsmenhomeimprovements.com</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>https://craftsmenhomeimprovements.com/roof-replacement-bloomington-mn/</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr"/>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>contact@chi-service.com</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>(952) 930-3777</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>Bloomington MN</t>
+        </is>
+      </c>
+      <c r="I148" t="n">
+        <v>86</v>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>roof replacement Bloomington MN</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 20:58 UTC (cycle 76)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L148"/>
+  <dimension ref="A1:L149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9039,7 +9039,6 @@
           <t>https://craftsmenhomeimprovements.com/roof-replacement-bloomington-mn/</t>
         </is>
       </c>
-      <c r="E148" t="inlineStr"/>
       <c r="F148" t="inlineStr">
         <is>
           <t>contact@chi-service.com</t>
@@ -9069,6 +9068,66 @@
         </is>
       </c>
       <c r="L148" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Precision Climate Control</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>yourairpro.com</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>https://yourairpro.com/heat-pump-services/</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Missouri Homes</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>info@yourairpro.com</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>636.293.2119</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>St Charles MO</t>
+        </is>
+      </c>
+      <c r="I149" t="n">
+        <v>90</v>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>heat pump installation St Charles MO</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 20:59 UTC (cycle 77)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L149"/>
+  <dimension ref="A1:L151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9133,6 +9133,126 @@
         </is>
       </c>
     </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Miami Metal Roofing</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>miami-metal-roofing.com</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>https://miami-metal-roofing.com/</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Standing Seam</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>info@miami-metal-roofing.com</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>(786) 628-0789</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>Miami FL</t>
+        </is>
+      </c>
+      <c r="I150" t="n">
+        <v>100</v>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Miami FL</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Proper Roofing</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>properoofing.com</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>https://properoofing.com/services/metal-roof/</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Proper Roofing</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>appointment@properoofing.com</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>786-999-5353</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>Miami FL</t>
+        </is>
+      </c>
+      <c r="I151" t="n">
+        <v>90</v>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Miami FL</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 21:06 UTC (cycle 82)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L151"/>
+  <dimension ref="A1:L152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9253,6 +9253,62 @@
         </is>
       </c>
     </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Sewer Services - Lakeland FL - Sparkman Plumbing Inc.</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>sparkmanplumbing.com</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>https://www.sparkmanplumbing.com/sewer</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr"/>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>bsparky@verizon.net</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>863-647-5765</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>Lakeland FL</t>
+        </is>
+      </c>
+      <c r="I152" t="n">
+        <v>92</v>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>sewer repair Lakeland FL</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 21:12 UTC (cycle 86)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L152"/>
+  <dimension ref="A1:L153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9274,7 +9274,6 @@
           <t>https://www.sparkmanplumbing.com/sewer</t>
         </is>
       </c>
-      <c r="E152" t="inlineStr"/>
       <c r="F152" t="inlineStr">
         <is>
           <t>bsparky@verizon.net</t>
@@ -9304,6 +9303,66 @@
         </is>
       </c>
       <c r="L152" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Home - Wayside Plumbing</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>wayside-plumbing.com</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>https://www.wayside-plumbing.com</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Rapid City</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>brandon@wayside-plumbing.com</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>(605) 939-8896</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>Rapid City SD</t>
+        </is>
+      </c>
+      <c r="I153" t="n">
+        <v>72</v>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>plumbing company Rapid City SD</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 21:25 UTC (cycle 95)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L153"/>
+  <dimension ref="A1:L154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9368,6 +9368,66 @@
         </is>
       </c>
     </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Sioux Falls Roofs Pro</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>siouxfallsroofs.com</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>https://siouxfallsroofs.com/</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Sun Valley</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>thorsonconstruction@gmail.com</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>(605) 728-8533</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>Sioux Falls SD</t>
+        </is>
+      </c>
+      <c r="I154" t="n">
+        <v>100</v>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>roofing contractor Sioux Falls SD</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 21:37 UTC (cycle 103)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L154"/>
+  <dimension ref="A1:L155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9428,6 +9428,62 @@
         </is>
       </c>
     </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Charlotte Roofing Pros</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>charlotteroofingnc.com</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>https://charlotteroofingnc.com/</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Areas About</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>info@charlotteroofingpros.com</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr"/>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>Charlotte NC</t>
+        </is>
+      </c>
+      <c r="I155" t="n">
+        <v>76</v>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>roof replacement Charlotte NC</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 21:40 UTC (cycle 105)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L155"/>
+  <dimension ref="A1:L156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9459,7 +9459,6 @@
           <t>info@charlotteroofingpros.com</t>
         </is>
       </c>
-      <c r="G155" t="inlineStr"/>
       <c r="H155" t="inlineStr">
         <is>
           <t>Charlotte NC</t>
@@ -9479,6 +9478,66 @@
         </is>
       </c>
       <c r="L155" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Roanoke, Blacksburg, &amp; Christiansburg</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>blueridgeheatingandair.com</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>https://blueridgeheatingandair.com/ac-installation/</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Schedule Your</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>brhainstall@gmail.com</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>(540) 381-1137</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>Roanoke VA</t>
+        </is>
+      </c>
+      <c r="I156" t="n">
+        <v>100</v>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>AC installation Roanoke VA</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 21:43 UTC (cycle 107)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L156"/>
+  <dimension ref="A1:L157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9543,6 +9543,66 @@
         </is>
       </c>
     </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>ON TOP ROOFING LLC</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>ontoproofingmi.com</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>https://www.ontoproofingmi.com/services/roof-replacement/roof-replacement-ann-arbor-mi</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Livingston County</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>info@ontoproofingmi.com</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>(810) 588-3933</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>Ann Arbor MI</t>
+        </is>
+      </c>
+      <c r="I157" t="n">
+        <v>100</v>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>roof replacement Ann Arbor MI</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 21:44 UTC (cycle 108)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L157"/>
+  <dimension ref="A1:L159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9603,6 +9603,126 @@
         </is>
       </c>
     </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Savannah HVAC Services | Dean Custom Air</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>deancustomair.com</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>https://www.deancustomair.com/savannah--ga</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Custom Air</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>info@hvacweb.com</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>843-258-3694</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>Savannah GA</t>
+        </is>
+      </c>
+      <c r="I158" t="n">
+        <v>100</v>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>air conditioning repair Savannah GA</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Truficient Energy Solutions</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>truficient.com</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>https://truficient.com/heat-pump-replacement-richardson-tx/</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>North Richardson</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>info@truficient.com</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>214-238-4349</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>Richardson TX</t>
+        </is>
+      </c>
+      <c r="I159" t="n">
+        <v>90</v>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>heat pump installation Richardson TX</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 21:47 UTC (cycle 110)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L159"/>
+  <dimension ref="A1:L162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9723,6 +9723,186 @@
         </is>
       </c>
     </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Emergency Plumber Portland OR</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>pdxplumber.com</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>https://www.pdxplumber.com/services/emergency-plumbing</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Who We</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>hello@pdxplumber.com</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>(503) 351-6906</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>Portland OR</t>
+        </is>
+      </c>
+      <c r="I160" t="n">
+        <v>100</v>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>emergency plumber Portland OR</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Stone Ranch Construction</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>stoneranch.com</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>https://stoneranch.com/roofing/anaheim-ca/</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Ranch Construction</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>admin@stoneranch.com</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>(714) 790-9925</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>Anaheim CA</t>
+        </is>
+      </c>
+      <c r="I161" t="n">
+        <v>100</v>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>roof replacement Anaheim CA</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>My Way Roofing</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>mywayroofing.com</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>https://mywayroofing.com/service-areas/anaheim/</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>My Way</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>info@mywayroofing.com</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>866-357-9339</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>Anaheim CA</t>
+        </is>
+      </c>
+      <c r="I162" t="n">
+        <v>80</v>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>roof replacement Anaheim CA</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 21:50 UTC (cycle 112)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L162"/>
+  <dimension ref="A1:L164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9903,6 +9903,126 @@
         </is>
       </c>
     </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Bethlehem Roof Pros</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>bethlehemparoofpros.com</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>https://bethlehemparoofpros.com/</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>Bethlehem Roofing</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>quotes@bethlehemparoofpros.com</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>(610) 492-6917</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>Bethlehem PA</t>
+        </is>
+      </c>
+      <c r="I163" t="n">
+        <v>100</v>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>roof repair company Bethlehem PA</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>1 Source Roofing and Restoration</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>1sourceroofingandrestoration.com</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>https://1sourceroofingandrestoration.com/city-sandy-springs-ga.html</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Claims Assistance</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>info@1sourceroofingandrestoration.com</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>(404) 277-1377</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>Sandy Springs GA</t>
+        </is>
+      </c>
+      <c r="I164" t="n">
+        <v>90</v>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>roofing contractor Sandy Springs GA</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 22:01 UTC (cycle 119)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L164"/>
+  <dimension ref="A1:L165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10023,6 +10023,66 @@
         </is>
       </c>
     </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>CAN Roof Construction</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>canroofconstruction.com</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>https://canroofconstruction.com/</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Rated Roofing</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>info@canroofconstruction.com</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>(857) 415 7727</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>Boston MA</t>
+        </is>
+      </c>
+      <c r="I165" t="n">
+        <v>90</v>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>residential roofing company Boston MA</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 22:05 UTC (cycle 122)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L165"/>
+  <dimension ref="A1:L166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10083,6 +10083,62 @@
         </is>
       </c>
     </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Select Comfort Systems | West Valley City, UT</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>selectcomfortsystems.com</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>https://www.selectcomfortsystems.com/</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr"/>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>lisa@selectcomfortsystems.com</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>801-969-7088</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>West Valley City UT</t>
+        </is>
+      </c>
+      <c r="I166" t="n">
+        <v>100</v>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>heating and cooling company West Valley City UT</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 22:21 UTC (cycle 133)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L166"/>
+  <dimension ref="A1:L168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10104,7 +10104,6 @@
           <t>https://www.selectcomfortsystems.com/</t>
         </is>
       </c>
-      <c r="E166" t="inlineStr"/>
       <c r="F166" t="inlineStr">
         <is>
           <t>lisa@selectcomfortsystems.com</t>
@@ -10134,6 +10133,126 @@
         </is>
       </c>
       <c r="L166" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>HVAC Company New Jersey</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>heat-pump-installation-paterson.aeshvacnj.com</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>https://heat-pump-installation-paterson.aeshvacnj.com/</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Call Us</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>example@mail.com</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>(888) 978-1291</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>Paterson NJ</t>
+        </is>
+      </c>
+      <c r="I167" t="n">
+        <v>100</v>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>heat pump installation Paterson NJ</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Roof Repair Albany NY</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>roofrepairalbany.com</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>https://www.roofrepairalbany.com/</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Residential Roofing</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>roofrepairalbany@gmail.com</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>(518) 400-3908</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>Albany NY</t>
+        </is>
+      </c>
+      <c r="I168" t="n">
+        <v>100</v>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>roof repair company Albany NY</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L168" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 22:25 UTC (cycle 136)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L168"/>
+  <dimension ref="A1:L169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10258,6 +10258,62 @@
         </is>
       </c>
     </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>HVAC Services | W4 Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>w4heatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>https://www.w4heatingandcooling.com/</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr"/>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>w4heatingandcooling@gmail.com</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>(325) 762-6061</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>Abilene TX</t>
+        </is>
+      </c>
+      <c r="I169" t="n">
+        <v>100</v>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>heating and cooling company Abilene TX</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 22:33 UTC (cycle 141)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L169"/>
+  <dimension ref="A1:L170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10279,7 +10279,6 @@
           <t>https://www.w4heatingandcooling.com/</t>
         </is>
       </c>
-      <c r="E169" t="inlineStr"/>
       <c r="F169" t="inlineStr">
         <is>
           <t>w4heatingandcooling@gmail.com</t>
@@ -10309,6 +10308,66 @@
         </is>
       </c>
       <c r="L169" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>RJC Plumbing LLC</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>rjcplumbing.com</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>https://www.rjcplumbing.com/service-areas/lewiston/drain-cleaning</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Free Quote</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>rjcplumbing@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>(207) 549-0064</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>Lewiston ME</t>
+        </is>
+      </c>
+      <c r="I170" t="n">
+        <v>100</v>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>drain cleaning service Lewiston ME</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L170" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 22:36 UTC (cycle 143)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L170"/>
+  <dimension ref="A1:L171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10373,6 +10373,62 @@
         </is>
       </c>
     </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Plumber Anaheim | 60 Mins To You: Anaheim Plumber Champions</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>anaheimplumberchampions.com</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>http://anaheimplumberchampions.com/sewer-repair-anaheim-ca/</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr"/>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>service@anaheimplumberchampions.com</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>(714) 400-2048</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>Anaheim CA</t>
+        </is>
+      </c>
+      <c r="I171" t="n">
+        <v>88</v>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>sewer repair Anaheim CA</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 22:50 UTC (cycle 153)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L171"/>
+  <dimension ref="A1:L172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10394,7 +10394,6 @@
           <t>http://anaheimplumberchampions.com/sewer-repair-anaheim-ca/</t>
         </is>
       </c>
-      <c r="E171" t="inlineStr"/>
       <c r="F171" t="inlineStr">
         <is>
           <t>service@anaheimplumberchampions.com</t>
@@ -10424,6 +10423,66 @@
         </is>
       </c>
       <c r="L171" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Kindred Construction</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>kindredconstruct.com</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>https://kindredconstruct.com/amarillo/</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Tascosa Office</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>info@kindredconstruct.com</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>806-440-2167</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>Amarillo TX</t>
+        </is>
+      </c>
+      <c r="I172" t="n">
+        <v>100</v>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>roofing contractor Amarillo TX</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L172" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 22:52 UTC (cycle 154)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L172"/>
+  <dimension ref="A1:L173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10488,6 +10488,66 @@
         </is>
       </c>
     </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Qualitech Home Services</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>qualitechhomeservices.com</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>https://www.qualitechhomeservices.com/en/service-areas/miramar</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Homeowners What</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>qualitechhomeservices@gmail.com</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>(754) 326-9233</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>Miramar FL</t>
+        </is>
+      </c>
+      <c r="I173" t="n">
+        <v>90</v>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>roofer Miramar FL</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 22:53 UTC (cycle 155)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L173"/>
+  <dimension ref="A1:L175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10548,6 +10548,122 @@
         </is>
       </c>
     </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Fresh Air Solutions and Tech LLC</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>freshairsolutionsandtech.com</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>https://www.freshairsolutionsandtech.com/areas/fishers-in</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr"/>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>fastairquality@gmail.com</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>(317) 652-9835</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>Fishers IN</t>
+        </is>
+      </c>
+      <c r="I174" t="n">
+        <v>100</v>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>HVAC contractor Fishers IN</t>
+        </is>
+      </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>HVAC Fishers IN | JD's Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>jdsmechanical.com</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>https://jdsmechanical.com/fishers.html</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>Hamilton County</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>office@jdsheatingandair.com</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>(317) 413-9303</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>Fishers IN</t>
+        </is>
+      </c>
+      <c r="I175" t="n">
+        <v>88</v>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>HVAC contractor Fishers IN</t>
+        </is>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 22:55 UTC (cycle 156)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L175"/>
+  <dimension ref="A1:L176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10569,7 +10569,6 @@
           <t>https://www.freshairsolutionsandtech.com/areas/fishers-in</t>
         </is>
       </c>
-      <c r="E174" t="inlineStr"/>
       <c r="F174" t="inlineStr">
         <is>
           <t>fastairquality@gmail.com</t>
@@ -10659,6 +10658,66 @@
         </is>
       </c>
       <c r="L175" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>A Better Roofing Company</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>abetterroofing.com</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>https://www.abetterroofing.com/</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Posts Clear</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>abr@abetterroofing.com</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>(206) 935-1575</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>Seattle WA</t>
+        </is>
+      </c>
+      <c r="I176" t="n">
+        <v>100</v>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>roof replacement Seattle WA</t>
+        </is>
+      </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L176" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 23:09 UTC (cycle 166)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L176"/>
+  <dimension ref="A1:L177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10723,6 +10723,66 @@
         </is>
       </c>
     </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Pomykal Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>gopomykal.com</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>https://gopomykal.com/service-area/hvac-services-killeen-tx/</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>At Pomykal</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>gopomykal@gmail.com</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>254-938-6290</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>Killeen TX</t>
+        </is>
+      </c>
+      <c r="I177" t="n">
+        <v>90</v>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>heating and cooling company Killeen TX</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 23:11 UTC (cycle 167)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L177"/>
+  <dimension ref="A1:L178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10783,6 +10783,62 @@
         </is>
       </c>
     </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>TNT ROOFING LAS VEGAS</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>tntroofinglasvegas.com</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>https://tntroofinglasvegas.com/</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr"/>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>tntroofing.lasvegas@gmail.com</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>702 220-4496</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="I178" t="n">
+        <v>90</v>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>roofer Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 23:12 UTC (cycle 168)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L178"/>
+  <dimension ref="A1:L179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10804,7 +10804,6 @@
           <t>https://tntroofinglasvegas.com/</t>
         </is>
       </c>
-      <c r="E178" t="inlineStr"/>
       <c r="F178" t="inlineStr">
         <is>
           <t>tntroofing.lasvegas@gmail.com</t>
@@ -10834,6 +10833,66 @@
         </is>
       </c>
       <c r="L178" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Roofing Contractor in Fayetteville, NC | GAF Master Elite | Roof Methods</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>roofmethods.com</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>https://roofmethods.com/areas-served/fayetteville-nc</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Business Hours</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>roofmethods@gmail.com</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>(910) 399-6123</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>Fayetteville NC</t>
+        </is>
+      </c>
+      <c r="I179" t="n">
+        <v>90</v>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>roof replacement Fayetteville NC</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 23:15 UTC (cycle 170)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L179"/>
+  <dimension ref="A1:L180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10898,6 +10898,66 @@
         </is>
       </c>
     </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>KP Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>kphvac.com</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>https://kphvac.com/</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Rick Peterson</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>rick@kphvac.com</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>920.687.2665</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>Appleton WI</t>
+        </is>
+      </c>
+      <c r="I180" t="n">
+        <v>90</v>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>HVAC contractor Appleton WI</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 23:26 UTC (cycle 177)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L180"/>
+  <dimension ref="A1:L182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10958,6 +10958,118 @@
         </is>
       </c>
     </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Slopes Roofing &amp; Construction</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>slopesroofing.com</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>https://slopesroofing.com/service-areas/lake-charles</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr"/>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>jason@slopesroofing.com</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>(337) 718-6407</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>Lake Charles LA</t>
+        </is>
+      </c>
+      <c r="I181" t="n">
+        <v>100</v>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>roof replacement Lake Charles LA</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>HVAC Contractor Boston | Canton | Northeastern Mechanical</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>northeasternmech.com</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>https://www.northeasternmech.com/</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr"/>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>sales@northeasternmech.com</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>(617) 394-1010</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>Boston MA</t>
+        </is>
+      </c>
+      <c r="I182" t="n">
+        <v>74</v>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>HVAC contractor Boston MA</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-26 23:40 UTC (cycle 187)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L182"/>
+  <dimension ref="A1:L183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10979,7 +10979,6 @@
           <t>https://slopesroofing.com/service-areas/lake-charles</t>
         </is>
       </c>
-      <c r="E181" t="inlineStr"/>
       <c r="F181" t="inlineStr">
         <is>
           <t>jason@slopesroofing.com</t>
@@ -11035,7 +11034,6 @@
           <t>https://www.northeasternmech.com/</t>
         </is>
       </c>
-      <c r="E182" t="inlineStr"/>
       <c r="F182" t="inlineStr">
         <is>
           <t>sales@northeasternmech.com</t>
@@ -11065,6 +11063,62 @@
         </is>
       </c>
       <c r="L182" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Drain Cleaning | Lancaster, PA | Valley Sewer Company LLC</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>valleysewerco.com</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>https://www.valleysewerco.com/contact/drain-cleaning-service-area/lancaster-pa</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr"/>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>valleysewerco@gmail.com</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>(717) 584-4445</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>Lancaster PA</t>
+        </is>
+      </c>
+      <c r="I183" t="n">
+        <v>90</v>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>drain cleaning service Lancaster PA</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-26 23:49 UTC (cycle 193)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-26.xlsx
+++ b/output/leads_2026-09-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L183"/>
+  <dimension ref="A1:L185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -11089,7 +11089,6 @@
           <t>https://www.valleysewerco.com/contact/drain-cleaning-service-area/lancaster-pa</t>
         </is>
       </c>
-      <c r="E183" t="inlineStr"/>
       <c r="F183" t="inlineStr">
         <is>
           <t>valleysewerco@gmail.com</t>
@@ -11119,6 +11118,126 @@
         </is>
       </c>
       <c r="L183" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Earl W. Johnston Roofing, LLC</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>johnstonroofing.com</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>https://johnstonroofing.com/service-areas/pembroke-pines-fl/</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Better Business</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>info@johnstonroofing.com</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>(954) 989-7794</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>Pembroke Pines FL</t>
+        </is>
+      </c>
+      <c r="I184" t="n">
+        <v>100</v>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>residential roofing company Pembroke Pines FL</t>
+        </is>
+      </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Sniper Roofing LLC</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>sniperroofingllc.com</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>https://sniperroofingllc.com/</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Sniper Roofing</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>sniperroofing2025@gmail.com</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>(214) 770-4130</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>Corpus Christi TX</t>
+        </is>
+      </c>
+      <c r="I185" t="n">
+        <v>90</v>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>roofing contractor Corpus Christi TX</t>
+        </is>
+      </c>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L185" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>

</xml_diff>